<commit_message>
Add grants realisation row to Design Capital "Years realisation"
- Added a new row in the design-capital file "Years Realisation" field (placed directly below Grant percentage)

- This row is used to calculate grants realisation in the financial statements

- Supports grants realisation both in absolute values and as a percentage of CAPEX
</commit_message>
<xml_diff>
--- a/backend/Rwanda/design-capital-Aligned.xlsx
+++ b/backend/Rwanda/design-capital-Aligned.xlsx
@@ -8,21 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/Rwanda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_BA5CDC726F815813957798D5D86865518C81A08F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5803B468-542A-4082-8ED9-97D68734BA2B}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_BA5CDC726F815813957798D5D86865518C81A08F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3458181C-9ABF-4D58-AAD8-F0BF16568FE1}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity &amp; E-Cooking" sheetId="1" r:id="rId1"/>
     <sheet name="Electricity (Low access)" sheetId="2" r:id="rId2"/>
     <sheet name="LPG" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterate="1"/>
+  <calcPr calcId="191029" iterate="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="33">
   <si>
     <t>Units</t>
   </si>
@@ -118,6 +131,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Years realisation</t>
   </si>
 </sst>
 </file>
@@ -348,6 +364,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -667,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.54296875" customWidth="1"/>
@@ -838,61 +858,59 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A6" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="15">
-        <v>8</v>
+      <c r="B6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>3</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>3</v>
@@ -933,13 +951,13 @@
     </row>
     <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7" s="15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
@@ -980,60 +998,60 @@
     </row>
     <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="15">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>3</v>
+      <c r="B9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="15">
+        <v>25</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>3</v>
@@ -1073,438 +1091,438 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A11" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B11" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="24">
+      <c r="C11" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="24">
         <v>2023</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E11" s="24">
         <v>2024</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F11" s="24">
         <v>2025</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G11" s="24">
         <v>2026</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H11" s="24">
         <v>2027</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I11" s="24">
         <v>2028</v>
       </c>
-      <c r="J10" s="24">
+      <c r="J11" s="24">
         <v>2029</v>
       </c>
-      <c r="K10" s="24">
+      <c r="K11" s="24">
         <v>2030</v>
       </c>
-      <c r="L10" s="24">
+      <c r="L11" s="24">
         <v>2031</v>
       </c>
-      <c r="M10" s="24">
+      <c r="M11" s="24">
         <v>2032</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N11" s="24">
         <v>2033</v>
       </c>
-      <c r="O10" s="24">
+      <c r="O11" s="24">
         <v>2034</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="L11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="M11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="N11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="O11" s="25" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="M12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="N12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="O12" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B13" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D13" s="15">
         <v>368.58986301369862</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E13" s="15">
         <v>458.85931506849317</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F13" s="15">
         <v>469.89246575342469</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G13" s="15">
         <v>481.18178082191781</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H13" s="15">
         <v>492.18438356164381</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I13" s="15">
         <v>502.94041095890412</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J13" s="15">
         <v>543.94136986301373</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K13" s="15">
         <v>579.44602739726031</v>
       </c>
-      <c r="L12" s="15">
+      <c r="L13" s="15">
         <v>580.0302739726028</v>
       </c>
-      <c r="M12" s="15">
+      <c r="M13" s="15">
         <v>579.89671232876719</v>
       </c>
-      <c r="N12" s="15">
+      <c r="N13" s="15">
         <v>579.72315068493151</v>
       </c>
-      <c r="O12" s="15">
+      <c r="O13" s="15">
         <v>469.96794520547951</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="J13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="K13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="N13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="O13" s="20" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="J14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="18">
+      <c r="C15" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="18">
         <v>2023</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E15" s="18">
         <v>2024</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F15" s="18">
         <v>2025</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G15" s="18">
         <v>2026</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H15" s="18">
         <v>2027</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I15" s="18">
         <v>2028</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J15" s="18">
         <v>2029</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K15" s="18">
         <v>2030</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L15" s="18">
         <v>2031</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M15" s="18">
         <v>2032</v>
       </c>
-      <c r="N14" s="18">
+      <c r="N15" s="18">
         <v>2033</v>
       </c>
-      <c r="O14" s="18">
+      <c r="O15" s="18">
         <v>2034</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="15">
-        <v>0</v>
-      </c>
-      <c r="E15" s="15">
-        <v>0</v>
-      </c>
-      <c r="F15" s="15">
-        <v>0</v>
-      </c>
-      <c r="G15" s="15">
-        <v>0</v>
-      </c>
-      <c r="H15" s="15">
-        <v>0</v>
-      </c>
-      <c r="I15" s="15">
-        <v>0</v>
-      </c>
-      <c r="J15" s="15">
-        <v>0</v>
-      </c>
-      <c r="K15" s="15">
-        <v>0</v>
-      </c>
-      <c r="L15" s="15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="15">
-        <v>0</v>
-      </c>
-      <c r="N15" s="15">
-        <v>0</v>
-      </c>
-      <c r="O15" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.4">
-      <c r="A16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="N16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="O16" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+      <c r="D16" s="15">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15">
+        <v>0</v>
+      </c>
+      <c r="H16" s="15">
+        <v>0</v>
+      </c>
+      <c r="I16" s="15">
+        <v>0</v>
+      </c>
+      <c r="J16" s="15">
+        <v>0</v>
+      </c>
+      <c r="K16" s="15">
+        <v>0</v>
+      </c>
+      <c r="L16" s="15">
+        <v>0</v>
+      </c>
+      <c r="M16" s="15">
+        <v>0</v>
+      </c>
+      <c r="N16" s="15">
+        <v>0</v>
+      </c>
+      <c r="O16" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.4">
+      <c r="A17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="O17" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="B18" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="O17" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+      <c r="D18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C19" s="13">
         <v>6106.6536986301371</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O18" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="D19" s="7" t="s">
         <v>3</v>
       </c>
@@ -1543,62 +1561,62 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B21" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="15">
-        <v>1221.3307397260271</v>
-      </c>
       <c r="D21" s="7" t="s">
         <v>3</v>
       </c>
@@ -1620,7 +1638,7 @@
       <c r="J21" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="7" t="s">
@@ -1638,13 +1656,13 @@
     </row>
     <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="15">
-        <v>2931.1937753424659</v>
+        <v>1221.3307397260271</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>3</v>
@@ -1685,13 +1703,13 @@
     </row>
     <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="15">
-        <v>0</v>
+        <v>2931.1937753424659</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>3</v>
@@ -1714,7 +1732,7 @@
       <c r="J23" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L23" s="7" t="s">
@@ -1731,49 +1749,96 @@
       </c>
     </row>
     <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="15">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A25" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C25" s="13">
         <v>146.5596887671233</v>
       </c>
-      <c r="D24" t="s">
-        <v>3</v>
-      </c>
-      <c r="E24" t="s">
-        <v>3</v>
-      </c>
-      <c r="F24" t="s">
-        <v>3</v>
-      </c>
-      <c r="G24" t="s">
-        <v>3</v>
-      </c>
-      <c r="H24" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" t="s">
-        <v>3</v>
-      </c>
-      <c r="K24" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" t="s">
-        <v>3</v>
-      </c>
-      <c r="N24" t="s">
-        <v>3</v>
-      </c>
-      <c r="O24" t="s">
+      <c r="D25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25" t="s">
+        <v>3</v>
+      </c>
+      <c r="I25" t="s">
+        <v>3</v>
+      </c>
+      <c r="J25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" t="s">
+        <v>3</v>
+      </c>
+      <c r="N25" t="s">
+        <v>3</v>
+      </c>
+      <c r="O25" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1784,7 +1849,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.6328125" customWidth="1"/>
@@ -1956,61 +2021,59 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A6" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="15">
-        <v>8</v>
+      <c r="B6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>3</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>3</v>
@@ -2051,13 +2114,13 @@
     </row>
     <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7" s="15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
@@ -2098,60 +2161,60 @@
     </row>
     <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="15">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>3</v>
+      <c r="B9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="15">
+        <v>25</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>3</v>
@@ -2191,438 +2254,438 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A11" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B11" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="24">
+      <c r="C11" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="24">
         <v>2023</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E11" s="24">
         <v>2024</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F11" s="24">
         <v>2025</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G11" s="24">
         <v>2026</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H11" s="24">
         <v>2027</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I11" s="24">
         <v>2028</v>
       </c>
-      <c r="J10" s="24">
+      <c r="J11" s="24">
         <v>2029</v>
       </c>
-      <c r="K10" s="24">
+      <c r="K11" s="24">
         <v>2030</v>
       </c>
-      <c r="L10" s="24">
+      <c r="L11" s="24">
         <v>2031</v>
       </c>
-      <c r="M10" s="24">
+      <c r="M11" s="24">
         <v>2032</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N11" s="24">
         <v>2033</v>
       </c>
-      <c r="O10" s="24">
+      <c r="O11" s="24">
         <v>2034</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="L11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="M11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="N11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="O11" s="25" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="M12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="N12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="O12" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B13" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D13" s="15">
         <v>338.51090691555282</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E13" s="15">
         <v>408.4275048740443</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F13" s="15">
         <v>417.83372360437392</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G13" s="15">
         <v>427.49940323775081</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H13" s="15">
         <v>436.92998590609989</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I13" s="15">
         <v>446.12920698075823</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J13" s="15">
         <v>463.30843844446821</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K13" s="15">
         <v>476.22996902434608</v>
       </c>
-      <c r="L12" s="15">
+      <c r="L13" s="15">
         <v>477.63934740104207</v>
       </c>
-      <c r="M12" s="15">
+      <c r="M13" s="15">
         <v>478.50998209905072</v>
       </c>
-      <c r="N12" s="15">
+      <c r="N13" s="15">
         <v>479.31544016835869</v>
       </c>
-      <c r="O12" s="15">
+      <c r="O13" s="15">
         <v>402.47703859784559</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="J13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="K13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="N13" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="O13" s="20" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="J14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="O14" s="20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="18">
+      <c r="C15" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="18">
         <v>2023</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E15" s="18">
         <v>2024</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F15" s="18">
         <v>2025</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G15" s="18">
         <v>2026</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H15" s="18">
         <v>2027</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I15" s="18">
         <v>2028</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J15" s="18">
         <v>2029</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K15" s="18">
         <v>2030</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L15" s="18">
         <v>2031</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M15" s="18">
         <v>2032</v>
       </c>
-      <c r="N14" s="18">
+      <c r="N15" s="18">
         <v>2033</v>
       </c>
-      <c r="O14" s="18">
+      <c r="O15" s="18">
         <v>2034</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="15">
-        <v>0</v>
-      </c>
-      <c r="E15" s="15">
-        <v>0</v>
-      </c>
-      <c r="F15" s="15">
-        <v>0</v>
-      </c>
-      <c r="G15" s="15">
-        <v>0</v>
-      </c>
-      <c r="H15" s="15">
-        <v>0</v>
-      </c>
-      <c r="I15" s="15">
-        <v>0</v>
-      </c>
-      <c r="J15" s="15">
-        <v>0</v>
-      </c>
-      <c r="K15" s="15">
-        <v>0</v>
-      </c>
-      <c r="L15" s="15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="15">
-        <v>0</v>
-      </c>
-      <c r="N15" s="15">
-        <v>0</v>
-      </c>
-      <c r="O15" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.4">
-      <c r="A16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="N16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="O16" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+      <c r="D16" s="15">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15">
+        <v>0</v>
+      </c>
+      <c r="H16" s="15">
+        <v>0</v>
+      </c>
+      <c r="I16" s="15">
+        <v>0</v>
+      </c>
+      <c r="J16" s="15">
+        <v>0</v>
+      </c>
+      <c r="K16" s="15">
+        <v>0</v>
+      </c>
+      <c r="L16" s="15">
+        <v>0</v>
+      </c>
+      <c r="M16" s="15">
+        <v>0</v>
+      </c>
+      <c r="N16" s="15">
+        <v>0</v>
+      </c>
+      <c r="O16" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.4">
+      <c r="A17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="O17" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="B18" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="O17" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+      <c r="D18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C19" s="13">
         <v>5252.8109472536908</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O18" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="D19" s="7" t="s">
         <v>3</v>
       </c>
@@ -2661,62 +2724,62 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B21" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="15">
-        <v>1313.2027368134229</v>
-      </c>
       <c r="D21" s="7" t="s">
         <v>3</v>
       </c>
@@ -2738,7 +2801,7 @@
       <c r="J21" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="7" t="s">
@@ -2756,13 +2819,13 @@
     </row>
     <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="15">
-        <v>2626.4054736268458</v>
+        <v>1313.2027368134229</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>3</v>
@@ -2803,13 +2866,13 @@
     </row>
     <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C23" s="15">
-        <v>0</v>
+        <v>2626.4054736268458</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>3</v>
@@ -2832,7 +2895,7 @@
       <c r="J23" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L23" s="7" t="s">
@@ -2849,49 +2912,96 @@
       </c>
     </row>
     <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="15">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A25" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C25" s="13">
         <v>157.58432841761069</v>
       </c>
-      <c r="D24" t="s">
-        <v>3</v>
-      </c>
-      <c r="E24" t="s">
-        <v>3</v>
-      </c>
-      <c r="F24" t="s">
-        <v>3</v>
-      </c>
-      <c r="G24" t="s">
-        <v>3</v>
-      </c>
-      <c r="H24" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" t="s">
-        <v>3</v>
-      </c>
-      <c r="K24" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" t="s">
-        <v>3</v>
-      </c>
-      <c r="N24" t="s">
-        <v>3</v>
-      </c>
-      <c r="O24" t="s">
+      <c r="D25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25" t="s">
+        <v>3</v>
+      </c>
+      <c r="I25" t="s">
+        <v>3</v>
+      </c>
+      <c r="J25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" t="s">
+        <v>3</v>
+      </c>
+      <c r="N25" t="s">
+        <v>3</v>
+      </c>
+      <c r="O25" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2902,7 +3012,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="39.36328125" customWidth="1"/>
@@ -3074,61 +3184,59 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A6" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="15">
-        <v>8</v>
+      <c r="B6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>3</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>3</v>
@@ -3169,13 +3277,13 @@
     </row>
     <row r="7" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C7" s="15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
@@ -3216,60 +3324,60 @@
     </row>
     <row r="8" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A8" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="15">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>3</v>
+      <c r="B9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="15">
+        <v>25</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>3</v>
@@ -3309,438 +3417,438 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B11" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="18">
+      <c r="C11" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="18">
         <v>2023</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E11" s="18">
         <v>2024</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F11" s="18">
         <v>2025</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G11" s="18">
         <v>2026</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H11" s="18">
         <v>2027</v>
       </c>
-      <c r="I10" s="18">
+      <c r="I11" s="18">
         <v>2028</v>
       </c>
-      <c r="J10" s="18">
+      <c r="J11" s="18">
         <v>2029</v>
       </c>
-      <c r="K10" s="18">
+      <c r="K11" s="18">
         <v>2030</v>
       </c>
-      <c r="L10" s="18">
+      <c r="L11" s="18">
         <v>2031</v>
       </c>
-      <c r="M10" s="18">
+      <c r="M11" s="18">
         <v>2032</v>
       </c>
-      <c r="N10" s="18">
+      <c r="N11" s="18">
         <v>2033</v>
       </c>
-      <c r="O10" s="18">
+      <c r="O11" s="18">
         <v>2034</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="L11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="M11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="N11" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="O11" s="25" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="15">
-        <v>24.969972979147169</v>
-      </c>
-      <c r="E12" s="15">
-        <v>46.190535285009048</v>
-      </c>
-      <c r="F12" s="15">
-        <v>67.675764393030832</v>
-      </c>
-      <c r="G12" s="15">
-        <v>90.041275898114719</v>
-      </c>
-      <c r="H12" s="15">
-        <v>112.31833290568029</v>
-      </c>
-      <c r="I12" s="15">
-        <v>134.5082698326562</v>
-      </c>
-      <c r="J12" s="15">
-        <v>155.09976538117709</v>
-      </c>
-      <c r="K12" s="15">
-        <v>160.45690267578621</v>
-      </c>
-      <c r="L12" s="15">
-        <v>162.96314898733229</v>
-      </c>
-      <c r="M12" s="15">
-        <v>165.1953408959501</v>
-      </c>
-      <c r="N12" s="15">
-        <v>167.4223558913246</v>
-      </c>
-      <c r="O12" s="15">
-        <v>167.56558564262659</v>
+        <v>8</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="J12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="L12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="M12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="N12" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="O12" s="25" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="H13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="K13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="N13" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="O13" s="15" t="s">
-        <v>3</v>
+        <v>12</v>
+      </c>
+      <c r="D13" s="15">
+        <v>24.969972979147169</v>
+      </c>
+      <c r="E13" s="15">
+        <v>46.190535285009048</v>
+      </c>
+      <c r="F13" s="15">
+        <v>67.675764393030832</v>
+      </c>
+      <c r="G13" s="15">
+        <v>90.041275898114719</v>
+      </c>
+      <c r="H13" s="15">
+        <v>112.31833290568029</v>
+      </c>
+      <c r="I13" s="15">
+        <v>134.5082698326562</v>
+      </c>
+      <c r="J13" s="15">
+        <v>155.09976538117709</v>
+      </c>
+      <c r="K13" s="15">
+        <v>160.45690267578621</v>
+      </c>
+      <c r="L13" s="15">
+        <v>162.96314898733229</v>
+      </c>
+      <c r="M13" s="15">
+        <v>165.1953408959501</v>
+      </c>
+      <c r="N13" s="15">
+        <v>167.4223558913246</v>
+      </c>
+      <c r="O13" s="15">
+        <v>167.56558564262659</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="N14" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="O14" s="15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="18">
+      <c r="C15" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="18">
         <v>2023</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E15" s="18">
         <v>2024</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F15" s="18">
         <v>2025</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G15" s="18">
         <v>2026</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H15" s="18">
         <v>2027</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I15" s="18">
         <v>2028</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J15" s="18">
         <v>2029</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K15" s="18">
         <v>2030</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L15" s="18">
         <v>2031</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M15" s="18">
         <v>2032</v>
       </c>
-      <c r="N14" s="18">
+      <c r="N15" s="18">
         <v>2033</v>
       </c>
-      <c r="O14" s="18">
+      <c r="O15" s="18">
         <v>2034</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="15">
-        <v>0</v>
-      </c>
-      <c r="E15" s="15">
-        <v>0</v>
-      </c>
-      <c r="F15" s="15">
-        <v>0</v>
-      </c>
-      <c r="G15" s="15">
-        <v>0</v>
-      </c>
-      <c r="H15" s="15">
-        <v>0</v>
-      </c>
-      <c r="I15" s="15">
-        <v>0</v>
-      </c>
-      <c r="J15" s="15">
-        <v>0</v>
-      </c>
-      <c r="K15" s="15">
-        <v>0</v>
-      </c>
-      <c r="L15" s="15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="15">
-        <v>0</v>
-      </c>
-      <c r="N15" s="15">
-        <v>0</v>
-      </c>
-      <c r="O15" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.4">
-      <c r="A16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="K16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="N16" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="O16" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+      <c r="D16" s="15">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15">
+        <v>0</v>
+      </c>
+      <c r="H16" s="15">
+        <v>0</v>
+      </c>
+      <c r="I16" s="15">
+        <v>0</v>
+      </c>
+      <c r="J16" s="15">
+        <v>0</v>
+      </c>
+      <c r="K16" s="15">
+        <v>0</v>
+      </c>
+      <c r="L16" s="15">
+        <v>0</v>
+      </c>
+      <c r="M16" s="15">
+        <v>0</v>
+      </c>
+      <c r="N16" s="15">
+        <v>0</v>
+      </c>
+      <c r="O16" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="16" x14ac:dyDescent="0.4">
+      <c r="A17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="O17" s="14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="B18" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="O17" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+      <c r="D18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C19" s="13">
         <v>1456.407250767835</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O18" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="D19" s="7" t="s">
         <v>3</v>
       </c>
@@ -3779,62 +3887,62 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B21" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="15">
-        <v>582.56290030713399</v>
-      </c>
       <c r="D21" s="7" t="s">
         <v>3</v>
       </c>
@@ -3856,7 +3964,7 @@
       <c r="J21" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L21" s="7" t="s">
@@ -3874,13 +3982,13 @@
     </row>
     <row r="22" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="15">
-        <v>0</v>
+        <v>582.56290030713399</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>3</v>
@@ -3921,7 +4029,7 @@
     </row>
     <row r="23" spans="1:15" ht="16" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>12</v>
@@ -3950,7 +4058,7 @@
       <c r="J23" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="2" t="s">
         <v>3</v>
       </c>
       <c r="L23" s="7" t="s">
@@ -3967,49 +4075,96 @@
       </c>
     </row>
     <row r="24" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="15">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="16" x14ac:dyDescent="0.35">
+      <c r="A25" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C25" s="13">
         <v>69.907548036856085</v>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="N24" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O24" s="7" t="s">
+      <c r="D25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O25" s="7" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>